<commit_message>
Lot 3 : verification des fermetures, remplace 3 sites morts
Verifie les 35 prospects du lot 3 sur Google Maps : aucune fermeture
definitive. 3 domaines etaient toutefois morts (page d'erreur) alors que
les entreprises elles-memes restent actives - remplaces par des
prospects verifies (Ongles et Beaute a Bayonne, Salon Lumiere a Lyon,
Cycles et Passion a Bordeaux). Les 3 anciens domaines rejoignent
NOT_QUALIFIED_DOMAINS pour ne plus jamais ressortir.
</commit_message>
<xml_diff>
--- a/lot_03.xlsx
+++ b/lot_03.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,8 +92,20 @@
       <color rgb="00111827"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00374151"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +125,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F9FAFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -142,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -208,11 +230,17 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1073,39 +1101,39 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>fabien.coiffure.free.fr</t>
+          <t>alizebeaute.fr</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>Fabien Coiffure</t>
+          <t>Alizé beauté</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Brest</t>
+          <t>Bourges</t>
         </is>
       </c>
       <c r="D5" s="17" t="inlineStr"/>
       <c r="E5" s="18" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>18</t>
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="G5" s="18" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I5" s="19" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I5" s="22" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J5" s="20" t="inlineStr">
@@ -1115,30 +1143,30 @@
       </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (1) | doctype ancien | non responsive | document.write | pas de @media | px uniquement | pas de flex/grid | pas de variables CSS | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (2) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>alizebeaute.fr</t>
+          <t>b-gilles-coiffeur.fr</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Alizé beauté</t>
+          <t>B Gilles Coiffeur</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Bourges</t>
+          <t>Perpignan</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>66</t>
         </is>
       </c>
       <c r="F6" s="9" t="n">
@@ -1164,30 +1192,30 @@
       </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (2) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (3) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>b-gilles-coiffeur.fr</t>
+          <t>centrebeautedesarceaux.fr</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>B Gilles Coiffeur</t>
+          <t>Centre de beauté des Arceaux</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Perpignan</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D7" s="17" t="inlineStr"/>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>34</t>
         </is>
       </c>
       <c r="F7" s="9" t="n">
@@ -1213,30 +1241,34 @@
       </c>
       <c r="K7" s="21" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (3) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>centrebeautedesarceaux.fr</t>
+          <t>coiffure-eric-78.com</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Centre de beauté des Arceaux</t>
+          <t>Eric Coiffure</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Montpellier</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr"/>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>Versailles (78000)</t>
+        </is>
+      </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F8" s="9" t="n">
@@ -1262,34 +1294,30 @@
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (1) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (15) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>coiffure-eric-78.com</t>
+          <t>dupaty-opticien-rochelle.fr</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>Eric Coiffure</t>
+          <t>Optique Dupaty</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D9" s="23" t="inlineStr">
-        <is>
-          <t>Versailles (78000)</t>
-        </is>
-      </c>
+          <t>La Rochelle</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr"/>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
@@ -1315,30 +1343,30 @@
       </c>
       <c r="K9" s="21" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (15) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (3) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>dupaty-opticien-rochelle.fr</t>
+          <t>institut-beaute-belloceane.fr</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Optique Dupaty</t>
+          <t>Bellocéane</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>La Rochelle</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>75</t>
         </is>
       </c>
       <c r="F10" s="9" t="n">
@@ -1364,37 +1392,41 @@
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (3) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (13) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>institut-beaute-belloceane.fr</t>
+          <t>onglesbeaute.fr</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>Bellocéane</t>
+          <t>Ongles et Beauté</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D11" s="17" t="inlineStr"/>
+          <t>Bayonne</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>Saint-Jean-de-Luz (64500)</t>
+        </is>
+      </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="n">
-        <v>56</v>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="F11" s="25" t="n">
+        <v>37</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
@@ -1413,41 +1445,41 @@
       </c>
       <c r="K11" s="21" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (13) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>langebleu.fr</t>
+          <t>coiffeurhomme.com</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>L'Ange Bleu</t>
+          <t>Salon Lumière - Coiffure Hommes</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Caen</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr"/>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="n">
-        <v>56</v>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="n">
+        <v>28</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
+        <v>3</v>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
@@ -1462,7 +1494,7 @@
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>balises &lt;font&gt; (2) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (8) | bgcolor= | sans doctype | gif de mise en page | images .gif</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1824,7 @@
           <t>Dunkerque</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>Dunkerque (59140)</t>
         </is>
@@ -1845,7 +1877,7 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="24" t="inlineStr">
         <is>
           <t>Nanterre Envoyez (92000)</t>
         </is>
@@ -2257,7 +2289,7 @@
           <t>Lyon</t>
         </is>
       </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="D6" s="23" t="inlineStr">
         <is>
           <t>Miribel T (01700)</t>
         </is>
@@ -2359,7 +2391,7 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>Fontenay aux Roses (92260)</t>
         </is>
@@ -2571,7 +2603,7 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>DRAVEIL (91210)</t>
         </is>
@@ -2709,12 +2741,12 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>atbirvoyages.com</t>
+          <t>photo.rainbow.free.fr</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Atbir Voyages</t>
+          <t>Photo Rainbow</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -2729,10 +2761,10 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
@@ -2751,19 +2783,19 @@
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>layout en tableaux (4) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (3B) | aucun radius/ombre</t>
+          <t>layout en tableaux (7) | balises &lt;font&gt; (12) | &lt;marquee&gt; | bgcolor= | sans doctype | non responsive | images .gif</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>photo.rainbow.free.fr</t>
+          <t>accessrepro.fr</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>Photo Rainbow</t>
+          <t>Access Repro</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
@@ -2771,74 +2803,74 @@
           <t>Paris</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr"/>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>Saint Denis Mentions (93200)</t>
+        </is>
+      </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G9" s="18" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H9" s="19" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="I9" s="19" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="I9" s="22" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="J9" s="20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>wordpress 5.4.21</t>
         </is>
       </c>
       <c r="K9" s="21" t="inlineStr">
         <is>
-          <t>layout en tableaux (7) | balises &lt;font&gt; (12) | &lt;marquee&gt; | bgcolor= | sans doctype | non responsive | images .gif</t>
+          <t>layout en tableaux (3) | balises &lt;font&gt; (16) | doctype ancien | non responsive | pas de @media</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>accessrepro.fr</t>
+          <t>cyclesetpassion.fr</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Access Repro</t>
+          <t>Cycles et Passion</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
-        </is>
-      </c>
-      <c r="D10" s="24" t="inlineStr">
-        <is>
-          <t>Saint Denis Mentions (93200)</t>
-        </is>
-      </c>
+          <t>Bordeaux</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
+        <v>3</v>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
@@ -2848,12 +2880,12 @@
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>wordpress 5.4.21</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>layout en tableaux (3) | balises &lt;font&gt; (16) | doctype ancien | non responsive | pas de @media</t>
+          <t>balises &lt;font&gt; (9) | &lt;center&gt; | &lt;marquee&gt; | bgcolor= | doctype ancien | pas de @media | pas de flex/grid | pas de variables CSS</t>
         </is>
       </c>
     </row>

</xml_diff>